<commit_message>
feat: integra el bano y unifica compras y pedidos de corte del proyecto
</commit_message>
<xml_diff>
--- a/despiece-closet.xlsx
+++ b/despiece-closet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7e4bb88fb3ffb2f3/Desktop/proyecto_terraza/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="212" documentId="11_1010BCAFECFCD321D5BDC7783D3CA87A8D0287D7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E2B24E1-8AA9-4D62-B084-21B67B0E01C0}"/>
+  <xr:revisionPtr revIDLastSave="228" documentId="11_1010BCAFECFCD321D5BDC7783D3CA87A8D0287D7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5348D65A-8D40-4341-AEFE-74741A86B40C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="299">
   <si>
     <t>Clóset principal 195: despiece independiente</t>
   </si>
@@ -280,9 +280,6 @@
     <t>Pendiente plantilla</t>
   </si>
   <si>
-    <t>PROVISIONAL para corte: 2175 × 975, solape 30. Altura = hueco bajo el listón (2340−115) menos 50 mm del sistema. Sin perfil vertical en esta propuesta basada en el clóset del usuario. Confirmar taladros, altura, canto y suspensión. Tope conserva desfase de 50 mm entre hojas.</t>
-  </si>
-  <si>
     <t>C3-024</t>
   </si>
   <si>
@@ -316,9 +313,6 @@
     <t>Veta horizontal: frente de 824 de ancho, queda detrás de las hojas.</t>
   </si>
   <si>
-    <t>Cortar después de confirmar el kit Peralma (altura de hoja y plantilla).</t>
-  </si>
-  <si>
     <t>Supuestos por confirmar en la sucursal: Q2 cambia la medida que se pide; Q3 y Q4 marcan qué piezas pueden rechazar.</t>
   </si>
   <si>
@@ -838,12 +832,6 @@
     <t>Sucursal Madecentro</t>
   </si>
   <si>
-    <t>Confirmar con el kit Peralma FSCPCM20 la altura de hoja, la plantilla y la carga (hojas de ≈21,3 kg; el kit indica 30 kg: ¿por hoja o por kit?). Verificar si el tope amortiguado viene en el kit.</t>
-  </si>
-  <si>
-    <t>No cortar C3-023</t>
-  </si>
-  <si>
     <t>Proveedor del sistema</t>
   </si>
   <si>
@@ -926,6 +914,27 @@
   </si>
   <si>
     <t>Geometría del diseño.</t>
+  </si>
+  <si>
+    <t>Pedida 20 mm más alta (2195 en vez de 2175): en el armado, con el riel y los carros puestos, recortar el borde superior —tapado por la solapa— hasta que la guía inferior sujete la hoja. Nunca debe quedar corta.</t>
+  </si>
+  <si>
+    <t>Confirmar con el kit Peralma FSCPCM20 la carga (hojas de ≈21,3 kg; el kit indica 30 kg: ¿por hoja o por kit?) y si trae el tope amortiguado. La altura final de las hojas se ajusta en el armado.</t>
+  </si>
+  <si>
+    <t>Compra del kit; recorte de C3-023 en el armado</t>
+  </si>
+  <si>
+    <t>Hojas con sobremedida</t>
+  </si>
+  <si>
+    <t>Las hojas se piden de 2195 × 975 (20 mm más altas) y se recortan arriba en el armado, con el riel y los carros puestos, hasta que la guía inferior sujete la hoja. El borde recortado queda tapado por la solapa. La medida terminada de diseño sigue siendo 2175.</t>
+  </si>
+  <si>
+    <t>Decisión del usuario 27/10/2026</t>
+  </si>
+  <si>
+    <t>Medida terminada 2175 × 975, solape 30. Se pide de 2195 (20 mm más alta) y se recorta arriba en el armado, con el riel y los carros puestos, hasta que la guía inferior sujete la hoja; el borde recortado queda tapado por la solapa. Altura = hueco bajo el listón (2340−115) menos 50 mm del sistema. Sin perfil vertical, como el clóset del usuario. Tope conserva desfase de 50 mm entre hojas.</t>
   </si>
 </sst>
 </file>
@@ -1142,15 +1151,15 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1235,6 +1244,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2786,19 +2799,19 @@
       <c r="O29" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="P29" s="4" t="s">
-        <v>80</v>
+      <c r="P29" s="13" t="s">
+        <v>298</v>
       </c>
     </row>
     <row r="30" spans="1:16" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D30" s="1">
         <v>1</v>
@@ -2840,7 +2853,7 @@
         <v>25</v>
       </c>
       <c r="P30" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="31" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -2865,7 +2878,7 @@
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D32" s="1">
         <f>SUM(D7:D30)</f>
@@ -2874,7 +2887,7 @@
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
       <c r="G32" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H32" s="5">
         <f>SUM(H7:H30)</f>
@@ -2891,7 +2904,7 @@
     </row>
     <row r="33" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -2955,32 +2968,32 @@
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="S1" s="14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="P2" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="P2" s="17" t="s">
-        <v>89</v>
-      </c>
       <c r="Q2" s="18" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="S2" s="14" t="s">
         <v>19</v>
       </c>
       <c r="T2" s="14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="14" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="P3" s="17" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="Q3" s="26">
         <v>100</v>
@@ -2989,15 +3002,15 @@
         <v>56</v>
       </c>
       <c r="T3" s="14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="P4" s="17" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="Q4" s="26">
         <v>250</v>
@@ -3006,12 +3019,12 @@
         <v>76</v>
       </c>
       <c r="T4" s="14" t="s">
-        <v>92</v>
+        <v>292</v>
       </c>
     </row>
     <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="P5" s="17" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:20" ht="26.4" x14ac:dyDescent="0.25">
@@ -3019,43 +3032,43 @@
         <v>3</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C6" s="19" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="19" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E6" s="19" t="s">
         <v>6</v>
       </c>
       <c r="F6" s="19" t="s">
+        <v>94</v>
+      </c>
+      <c r="G6" s="19" t="s">
+        <v>95</v>
+      </c>
+      <c r="H6" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="G6" s="19" t="s">
+      <c r="I6" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="H6" s="19" t="s">
+      <c r="J6" s="19" t="s">
         <v>98</v>
       </c>
-      <c r="I6" s="19" t="s">
+      <c r="K6" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="J6" s="19" t="s">
+      <c r="L6" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="K6" s="19" t="s">
+      <c r="M6" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="L6" s="19" t="s">
+      <c r="N6" s="19" t="s">
         <v>102</v>
-      </c>
-      <c r="M6" s="19" t="s">
-        <v>103</v>
-      </c>
-      <c r="N6" s="19" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.25">
@@ -4334,7 +4347,7 @@
         <v>Si no la cantean: cortar a 479,1 × 79,1 y cantear en el armado.</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="26.4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A29" s="20" t="str">
         <f>Despiece!A29</f>
         <v>C3-023</v>
@@ -4356,8 +4369,8 @@
         <v>2</v>
       </c>
       <c r="F29" s="31">
-        <f>IF($Q$2="NO",ROUND(Despiece!M29,2),Despiece!E29)</f>
-        <v>2175</v>
+        <f>IF($Q$2="NO",ROUND(Despiece!M29,2),Despiece!E29)+20</f>
+        <v>2195</v>
       </c>
       <c r="G29" s="31">
         <f>IF($Q$2="NO",ROUND(Despiece!N29,2),Despiece!F29)</f>
@@ -4389,7 +4402,7 @@
       </c>
       <c r="N29" s="22" t="str">
         <f>IF(LEN(TRIM(IF($L29="Pequeña","Si no la cantean: cortar a "&amp;ROUND(Despiece!M29,2)&amp;" × "&amp;ROUND(Despiece!N29,2)&amp;" y cantear en el armado.","")&amp;" "&amp;IFERROR(VLOOKUP(Despiece!A29,$S$2:$T$40,2,FALSE),"")))=0,"—",TRIM(IF($L29="Pequeña","Si no la cantean: cortar a "&amp;ROUND(Despiece!M29,2)&amp;" × "&amp;ROUND(Despiece!N29,2)&amp;" y cantear en el armado.","")&amp;" "&amp;IFERROR(VLOOKUP(Despiece!A29,$S$2:$T$40,2,FALSE),"")))</f>
-        <v>Cortar después de confirmar el kit Peralma (altura de hoja y plantilla).</v>
+        <v>Pedida 20 mm más alta (2195 en vez de 2175): en el armado, con el riel y los carros puestos, recortar el borde superior —tapado por la solapa— hasta que la guía inferior sujete la hoja. Nunca debe quedar corta.</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
@@ -4452,20 +4465,20 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C32" s="16" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D32" s="23"/>
       <c r="E32" s="23"/>
       <c r="F32" s="16" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="G32" s="16" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="33" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C33" s="16" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D33" s="23"/>
       <c r="E33" s="23"/>
@@ -4480,7 +4493,7 @@
     </row>
     <row r="34" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C34" s="16" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D34" s="23"/>
       <c r="E34" s="23"/>
@@ -4495,7 +4508,7 @@
     </row>
     <row r="35" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C35" s="16" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D35" s="23"/>
       <c r="E35" s="23"/>
@@ -4510,20 +4523,20 @@
     </row>
     <row r="37" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C37" s="16" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="D37" s="23"/>
       <c r="E37" s="23"/>
       <c r="F37" s="16" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="38" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C38" s="14" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F38" s="27">
         <f>SUMPRODUCT(Despiece!$D$7:$D$30,(Despiece!$I$7:$I$30="2")+(Despiece!$J$7:$J$30="2")+(Despiece!$K$7:$K$30="2")+(Despiece!$L$7:$L$30="2"),--($L$7:$L$30="Pequeña"))</f>
@@ -4536,7 +4549,7 @@
     </row>
     <row r="39" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C39" s="14" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F39" s="28">
         <f>G33</f>
@@ -4549,7 +4562,7 @@
     </row>
     <row r="40" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C40" s="14" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F40" s="29">
         <v>0.1</v>
@@ -4560,7 +4573,7 @@
     </row>
     <row r="41" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C41" s="14" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F41" s="30">
         <v>0.2</v>
@@ -4571,7 +4584,7 @@
     </row>
     <row r="42" spans="3:14" x14ac:dyDescent="0.25">
       <c r="C42" s="16" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="D42" s="23"/>
       <c r="E42" s="23"/>
@@ -4585,31 +4598,31 @@
       </c>
     </row>
     <row r="43" spans="3:14" ht="49.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C43" s="38" t="s">
-        <v>242</v>
-      </c>
-      <c r="D43" s="39"/>
-      <c r="E43" s="39"/>
-      <c r="F43" s="39"/>
-      <c r="G43" s="39"/>
-      <c r="H43" s="39"/>
-      <c r="I43" s="39"/>
-      <c r="J43" s="39"/>
-      <c r="K43" s="39"/>
-      <c r="L43" s="39"/>
-      <c r="M43" s="39"/>
-      <c r="N43" s="39"/>
+      <c r="C43" s="39" t="s">
+        <v>240</v>
+      </c>
+      <c r="D43" s="40"/>
+      <c r="E43" s="40"/>
+      <c r="F43" s="40"/>
+      <c r="G43" s="40"/>
+      <c r="H43" s="40"/>
+      <c r="I43" s="40"/>
+      <c r="J43" s="40"/>
+      <c r="K43" s="40"/>
+      <c r="L43" s="40"/>
+      <c r="M43" s="40"/>
+      <c r="N43" s="40"/>
     </row>
     <row r="44" spans="3:14" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C44" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="F44" s="32"/>
       <c r="G44" s="32"/>
     </row>
     <row r="45" spans="3:14" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C45" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="F45" s="32">
         <v>0</v>
@@ -4620,7 +4633,7 @@
     </row>
     <row r="46" spans="3:14" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C46" s="33" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D46" s="33"/>
       <c r="E46" s="33"/>
@@ -4634,20 +4647,20 @@
       </c>
     </row>
     <row r="47" spans="3:14" ht="49.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C47" s="40" t="s">
-        <v>246</v>
-      </c>
-      <c r="D47" s="39"/>
-      <c r="E47" s="39"/>
-      <c r="F47" s="39"/>
-      <c r="G47" s="39"/>
-      <c r="H47" s="39"/>
-      <c r="I47" s="39"/>
-      <c r="J47" s="39"/>
-      <c r="K47" s="39"/>
-      <c r="L47" s="39"/>
-      <c r="M47" s="39"/>
-      <c r="N47" s="39"/>
+      <c r="C47" s="41" t="s">
+        <v>244</v>
+      </c>
+      <c r="D47" s="40"/>
+      <c r="E47" s="40"/>
+      <c r="F47" s="40"/>
+      <c r="G47" s="40"/>
+      <c r="H47" s="40"/>
+      <c r="I47" s="40"/>
+      <c r="J47" s="40"/>
+      <c r="K47" s="40"/>
+      <c r="L47" s="40"/>
+      <c r="M47" s="40"/>
+      <c r="N47" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4692,7 +4705,7 @@
     </row>
     <row r="2" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -4706,7 +4719,7 @@
     </row>
     <row r="3" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -4720,7 +4733,7 @@
     </row>
     <row r="4" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -4746,46 +4759,46 @@
     </row>
     <row r="6" spans="1:10" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>135</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>137</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>17</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C7" s="1">
         <v>5</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E7" s="9">
         <v>365872</v>
@@ -4795,29 +4808,29 @@
         <v>1829360</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="I7" s="12"/>
       <c r="J7" s="13" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C8" s="1">
         <f>Cantos!H7</f>
         <v>1</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E8" s="9">
         <v>531600</v>
@@ -4827,29 +4840,29 @@
         <v>531600</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="I8" s="1"/>
       <c r="J8" s="13" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C9" s="1">
         <f>Cantos!H8</f>
         <v>1</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E9" s="9">
         <v>285600</v>
@@ -4859,28 +4872,28 @@
         <v>285600</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="13" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C10" s="1">
         <v>3</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E10" s="9">
         <v>11287</v>
@@ -4890,28 +4903,28 @@
         <v>33861</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="H10" s="13" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="I10" s="12"/>
       <c r="J10" s="13" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C11" s="1">
         <v>1</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E11" s="9">
         <v>12730</v>
@@ -4921,28 +4934,28 @@
         <v>12730</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="4" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C12" s="1">
         <v>1</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E12" s="9">
         <v>33278</v>
@@ -4952,28 +4965,28 @@
         <v>33278</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C13" s="1">
         <v>2</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E13" s="9">
         <v>2743</v>
@@ -4983,26 +4996,26 @@
         <v>5486</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" s="1" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E14" s="9"/>
       <c r="F14" s="9" t="str">
@@ -5010,28 +5023,28 @@
         <v>Por cotizar</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="4" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C15" s="1">
         <v>3</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E15" s="9"/>
       <c r="F15" s="9" t="str">
@@ -5039,28 +5052,28 @@
         <v>Por cotizar</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="4" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C16" s="1">
         <v>6</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E16" s="9"/>
       <c r="F16" s="9" t="str">
@@ -5068,28 +5081,28 @@
         <v>Por cotizar</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="I16" s="1"/>
       <c r="J16" s="4" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C17" s="1">
         <v>6</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E17" s="9"/>
       <c r="F17" s="9" t="str">
@@ -5097,28 +5110,28 @@
         <v>Por cotizar</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="I17" s="1"/>
       <c r="J17" s="4" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C18" s="1">
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="E18" s="9"/>
       <c r="F18" s="9" t="str">
@@ -5126,28 +5139,28 @@
         <v>Por cotizar</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H18" s="13" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="I18" s="1"/>
       <c r="J18" s="4" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C19" s="1">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="E19" s="9"/>
       <c r="F19" s="9" t="str">
@@ -5155,28 +5168,28 @@
         <v>Por cotizar</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="4" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C20" s="1">
         <v>1</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="E20" s="9"/>
       <c r="F20" s="9" t="str">
@@ -5184,28 +5197,28 @@
         <v>Por cotizar</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="I20" s="1"/>
       <c r="J20" s="4" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C21" s="1">
         <v>1</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="E21" s="9"/>
       <c r="F21" s="9" t="str">
@@ -5213,19 +5226,19 @@
         <v>Por cotizar</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="I21" s="1"/>
       <c r="J21" s="4" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B22" s="10"/>
       <c r="C22" s="10"/>
@@ -5236,8 +5249,8 @@
         <v>2731915</v>
       </c>
       <c r="G22" s="10"/>
-      <c r="H22" s="41" t="s">
-        <v>294</v>
+      <c r="H22" s="38" t="s">
+        <v>290</v>
       </c>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
@@ -5299,7 +5312,7 @@
     </row>
     <row r="2" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -5308,7 +5321,7 @@
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="I2" s="1">
         <v>0.05</v>
@@ -5316,7 +5329,7 @@
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -5351,37 +5364,37 @@
     </row>
     <row r="6" spans="1:9" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="D6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="H6" s="3" t="s">
         <v>122</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>124</v>
       </c>
       <c r="I6" s="1"/>
     </row>
     <row r="7" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C7" s="8">
         <f>SUMPRODUCT(Despiece!$D$7:$D$30,Despiece!$E$7:$E$30,(Despiece!$I$7:$I$30="2")+(Despiece!$J$7:$J$30="2"))/1000+SUMPRODUCT(Despiece!$D$7:$D$30,Despiece!$F$7:$F$30,(Despiece!$K$7:$K$30="2")+(Despiece!$L$7:$L$30="2"))/1000</f>
@@ -5410,10 +5423,10 @@
     </row>
     <row r="8" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C8" s="8">
         <f>SUMPRODUCT(Despiece!$D$7:$D$30,Despiece!$E$7:$E$30,(Despiece!$I$7:$I$30="0.45")+(Despiece!$J$7:$J$30="0.45"))/1000+SUMPRODUCT(Despiece!$D$7:$D$30,Despiece!$F$7:$F$30,(Despiece!$K$7:$K$30="0.45")+(Despiece!$L$7:$L$30="0.45"))/1000</f>
@@ -5453,7 +5466,7 @@
     </row>
     <row r="10" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -5504,29 +5517,29 @@
   <sheetData>
     <row r="2" spans="1:5" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
+        <v>252</v>
+      </c>
+      <c r="B6" s="35" t="s">
+        <v>204</v>
+      </c>
+      <c r="C6" s="35" t="s">
+        <v>253</v>
+      </c>
+      <c r="D6" s="35" t="s">
         <v>254</v>
       </c>
-      <c r="B6" s="35" t="s">
-        <v>206</v>
-      </c>
-      <c r="C6" s="35" t="s">
+      <c r="E6" s="35" t="s">
         <v>255</v>
-      </c>
-      <c r="D6" s="35" t="s">
-        <v>256</v>
-      </c>
-      <c r="E6" s="35" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="26.4" x14ac:dyDescent="0.25">
@@ -5534,16 +5547,16 @@
         <v>1</v>
       </c>
       <c r="B7" s="37" t="s">
+        <v>256</v>
+      </c>
+      <c r="C7" s="37" t="s">
+        <v>257</v>
+      </c>
+      <c r="D7" s="37" t="s">
         <v>258</v>
       </c>
-      <c r="C7" s="37" t="s">
+      <c r="E7" s="37" t="s">
         <v>259</v>
-      </c>
-      <c r="D7" s="37" t="s">
-        <v>260</v>
-      </c>
-      <c r="E7" s="37" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="26.4" x14ac:dyDescent="0.25">
@@ -5551,16 +5564,16 @@
         <v>2</v>
       </c>
       <c r="B8" s="37" t="s">
+        <v>260</v>
+      </c>
+      <c r="C8" s="37" t="s">
+        <v>261</v>
+      </c>
+      <c r="D8" s="37" t="s">
         <v>262</v>
       </c>
-      <c r="C8" s="37" t="s">
+      <c r="E8" s="37" t="s">
         <v>263</v>
-      </c>
-      <c r="D8" s="37" t="s">
-        <v>264</v>
-      </c>
-      <c r="E8" s="37" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="26.4" x14ac:dyDescent="0.25">
@@ -5568,16 +5581,16 @@
         <v>3</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C9" s="37" t="s">
-        <v>266</v>
+        <v>293</v>
       </c>
       <c r="D9" s="37" t="s">
-        <v>267</v>
+        <v>294</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="26.4" x14ac:dyDescent="0.25">
@@ -5585,16 +5598,16 @@
         <v>4</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="D10" s="37" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -5602,16 +5615,16 @@
         <v>5</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="D11" s="37" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="26.4" x14ac:dyDescent="0.25">
@@ -5619,16 +5632,16 @@
         <v>6</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="D12" s="37" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="26.4" x14ac:dyDescent="0.25">
@@ -5636,16 +5649,16 @@
         <v>7</v>
       </c>
       <c r="B13" s="37" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C13" s="37" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="D13" s="37" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="E13" s="37" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="26.4" x14ac:dyDescent="0.25">
@@ -5653,16 +5666,16 @@
         <v>8</v>
       </c>
       <c r="B14" s="37" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="C14" s="37" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="D14" s="37" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="E14" s="37" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
     </row>
   </sheetData>
@@ -5672,7 +5685,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{056A28ED-57E4-401D-9DBD-33391A6C79EA}">
-  <dimension ref="A2:C15"/>
+  <dimension ref="A2:C16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.77734375" customWidth="1"/>
@@ -5682,122 +5695,133 @@
   <sheetData>
     <row r="2" spans="1:3" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B6" s="35" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="C6" s="35" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="37" t="s">
+        <v>205</v>
+      </c>
+      <c r="B7" s="37" t="s">
+        <v>206</v>
+      </c>
+      <c r="C7" s="37" t="s">
         <v>207</v>
-      </c>
-      <c r="B7" s="37" t="s">
-        <v>208</v>
-      </c>
-      <c r="C7" s="37" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A8" s="37" t="s">
+        <v>208</v>
+      </c>
+      <c r="B8" s="37" t="s">
+        <v>209</v>
+      </c>
+      <c r="C8" s="37" t="s">
         <v>210</v>
-      </c>
-      <c r="B8" s="37" t="s">
-        <v>211</v>
-      </c>
-      <c r="C8" s="37" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A9" s="37" t="s">
+        <v>211</v>
+      </c>
+      <c r="B9" s="37" t="s">
+        <v>212</v>
+      </c>
+      <c r="C9" s="37" t="s">
         <v>213</v>
-      </c>
-      <c r="B9" s="37" t="s">
-        <v>214</v>
-      </c>
-      <c r="C9" s="37" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A10" s="37" t="s">
+        <v>214</v>
+      </c>
+      <c r="B10" s="37" t="s">
+        <v>215</v>
+      </c>
+      <c r="C10" s="37" t="s">
         <v>216</v>
-      </c>
-      <c r="B10" s="37" t="s">
-        <v>217</v>
-      </c>
-      <c r="C10" s="37" t="s">
-        <v>218</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A11" s="37" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C11" s="37" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A12" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="B12" s="37" t="s">
+        <v>220</v>
+      </c>
+      <c r="C12" s="37" t="s">
         <v>221</v>
-      </c>
-      <c r="B12" s="37" t="s">
-        <v>222</v>
-      </c>
-      <c r="C12" s="37" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A13" s="37" t="s">
+        <v>222</v>
+      </c>
+      <c r="B13" s="37" t="s">
+        <v>223</v>
+      </c>
+      <c r="C13" s="37" t="s">
         <v>224</v>
-      </c>
-      <c r="B13" s="37" t="s">
-        <v>225</v>
-      </c>
-      <c r="C13" s="37" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A14" s="37" t="s">
+        <v>226</v>
+      </c>
+      <c r="B14" s="37" t="s">
+        <v>227</v>
+      </c>
+      <c r="C14" s="37" t="s">
         <v>228</v>
-      </c>
-      <c r="B14" s="37" t="s">
-        <v>229</v>
-      </c>
-      <c r="C14" s="37" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A15" s="37" t="s">
+        <v>230</v>
+      </c>
+      <c r="B15" s="37" t="s">
+        <v>231</v>
+      </c>
+      <c r="C15" s="37" t="s">
         <v>232</v>
       </c>
-      <c r="B15" s="37" t="s">
-        <v>233</v>
-      </c>
-      <c r="C15" s="37" t="s">
-        <v>234</v>
+    </row>
+    <row r="16" spans="1:3" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A16" s="37" t="s">
+        <v>295</v>
+      </c>
+      <c r="B16" s="37" t="s">
+        <v>296</v>
+      </c>
+      <c r="C16" s="37" t="s">
+        <v>297</v>
       </c>
     </row>
   </sheetData>

</xml_diff>